<commit_message>
Atualizar sistema de loterias com dados reais - incluir concurso 3030 da Mega-Sena e configurar atualização automática
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
+++ b/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
@@ -413,14 +413,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
+        <v>2414</v>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>2413</v>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>

</xml_diff>

<commit_message>
Atualizar todas as loterias até 19/07 - concursos mais recentes adicionados
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
+++ b/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
@@ -413,28 +413,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
+        <v>2416</v>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C1" t="n">
+        <v>17</v>
+      </c>
+      <c r="D1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1" t="n">
+        <v>36</v>
+      </c>
+      <c r="F1" t="n">
+        <v>50</v>
+      </c>
+      <c r="G1" t="n">
+        <v>70</v>
+      </c>
+      <c r="H1" t="n">
+        <v>74</v>
+      </c>
+      <c r="I1" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>2414</v>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>2413</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualizar resultados das loterias - 07/08/2026
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
+++ b/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
@@ -413,64 +413,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
+        <v>2425</v>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1" t="n">
+        <v>41</v>
+      </c>
+      <c r="F1" t="n">
+        <v>52</v>
+      </c>
+      <c r="G1" t="n">
+        <v>60</v>
+      </c>
+      <c r="H1" t="n">
+        <v>62</v>
+      </c>
+      <c r="I1" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>2416</v>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="C1" t="n">
+      <c r="C2" t="n">
         <v>17</v>
       </c>
-      <c r="D1" t="n">
+      <c r="D2" t="n">
         <v>30</v>
       </c>
-      <c r="E1" t="n">
+      <c r="E2" t="n">
         <v>36</v>
       </c>
-      <c r="F1" t="n">
+      <c r="F2" t="n">
         <v>50</v>
       </c>
-      <c r="G1" t="n">
+      <c r="G2" t="n">
         <v>70</v>
       </c>
-      <c r="H1" t="n">
+      <c r="H2" t="n">
         <v>74</v>
       </c>
-      <c r="I1" t="n">
+      <c r="I2" t="n">
         <v>77</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>2414</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2413</v>
+        <v>2414</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -481,6 +495,23 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2413</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizar dados das loterias até 21/08/2026 - novos concursos adicionados
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
+++ b/historicoresultadosloteriasnacionais/timemania_asloterias.xlsx
@@ -413,95 +413,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
+        <v>2431</v>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C1" t="n">
+        <v>18</v>
+      </c>
+      <c r="D1" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1" t="n">
+        <v>55</v>
+      </c>
+      <c r="F1" t="n">
+        <v>58</v>
+      </c>
+      <c r="G1" t="n">
+        <v>63</v>
+      </c>
+      <c r="H1" t="n">
+        <v>65</v>
+      </c>
+      <c r="I1" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>2425</v>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="C1" t="n">
+      <c r="C2" t="n">
         <v>8</v>
       </c>
-      <c r="D1" t="n">
+      <c r="D2" t="n">
         <v>22</v>
       </c>
-      <c r="E1" t="n">
+      <c r="E2" t="n">
         <v>41</v>
       </c>
-      <c r="F1" t="n">
+      <c r="F2" t="n">
         <v>52</v>
       </c>
-      <c r="G1" t="n">
+      <c r="G2" t="n">
         <v>60</v>
       </c>
-      <c r="H1" t="n">
+      <c r="H2" t="n">
         <v>62</v>
       </c>
-      <c r="I1" t="n">
+      <c r="I2" t="n">
         <v>67</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>2416</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C3" t="n">
         <v>17</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D3" t="n">
         <v>30</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E3" t="n">
         <v>36</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F3" t="n">
         <v>50</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G3" t="n">
         <v>70</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H3" t="n">
         <v>74</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I3" t="n">
         <v>77</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2414</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2413</v>
+        <v>2414</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -512,6 +526,23 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2413</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>